<commit_message>
Changed column names to indicator names instead of codes and also added another column log_gdp_pc that normalizes gdp_pc values by taking natural log
</commit_message>
<xml_diff>
--- a/RAW_DATA_XLSX/BGD_raw_data.xlsx
+++ b/RAW_DATA_XLSX/BGD_raw_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,52 +429,57 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>BX.KLT.DINV.WD.GD.ZS</t>
+          <t>education</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>FP.CPI.TOTL.ZG</t>
+          <t>fdi</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>NE.TRD.GNFS.ZS</t>
+          <t>gdp_growth</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>NV.IND.TOTL.ZS</t>
+          <t>gdp_pc</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>NY.GDP.MKTP.KD.ZG</t>
+          <t>log_gdp_pc</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>NY.GDP.PCAP.KD</t>
+          <t>gini</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>SE.SEC.ENRR</t>
+          <t>industry</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>SI.POV.GINI</t>
+          <t>inflation</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>SL.UEM.TOTL.ZS</t>
+          <t>trade</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>SP.URB.TOTL.IN.ZS</t>
+          <t>unemployment</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>urban</t>
         </is>
       </c>
     </row>
@@ -487,32 +492,35 @@
       <c r="B2" t="n">
         <v>1995</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
         <v>0.00499837818821925</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
+        <v>5.12127789724337</v>
+      </c>
+      <c r="F2" t="n">
+        <v>537.931946643983</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6.287732058934044</v>
+      </c>
+      <c r="H2" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="I2" t="n">
+        <v>23.5808244521571</v>
+      </c>
+      <c r="J2" t="n">
         <v>10.2978117947206</v>
       </c>
-      <c r="E2" t="n">
+      <c r="K2" t="n">
         <v>28.2094960764218</v>
       </c>
-      <c r="F2" t="n">
-        <v>23.5808244521571</v>
-      </c>
-      <c r="G2" t="n">
-        <v>5.12127789724337</v>
-      </c>
-      <c r="H2" t="n">
-        <v>537.931946643983</v>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>2.441</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>21.661231550566</v>
       </c>
     </row>
@@ -525,30 +533,33 @@
       <c r="B3" t="n">
         <v>1996</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
         <v>0.0291349551912919</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
+        <v>4.52291921684423</v>
+      </c>
+      <c r="F3" t="n">
+        <v>552.077107138767</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6.313687723367389</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>21.6839165728619</v>
+      </c>
+      <c r="J3" t="n">
         <v>2.37712902953223</v>
       </c>
-      <c r="E3" t="n">
+      <c r="K3" t="n">
         <v>26.0760877233809</v>
       </c>
-      <c r="F3" t="n">
-        <v>21.6839165728619</v>
-      </c>
-      <c r="G3" t="n">
-        <v>4.52291921684423</v>
-      </c>
-      <c r="H3" t="n">
-        <v>552.077107138767</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>2.51</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>21.9780786680138</v>
       </c>
     </row>
@@ -561,30 +572,33 @@
       <c r="B4" t="n">
         <v>1997</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="n">
         <v>0.288896567530213</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
+        <v>4.4898964976265</v>
+      </c>
+      <c r="F4" t="n">
+        <v>566.271140847632</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6.339073010930571</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>21.8626700944451</v>
+      </c>
+      <c r="J4" t="n">
         <v>5.30560105668801</v>
       </c>
-      <c r="E4" t="n">
+      <c r="K4" t="n">
         <v>26.3255133900833</v>
       </c>
-      <c r="F4" t="n">
-        <v>21.8626700944451</v>
-      </c>
-      <c r="G4" t="n">
-        <v>4.4898964976265</v>
-      </c>
-      <c r="H4" t="n">
-        <v>566.271140847632</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>2.698</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>22.2953437419401</v>
       </c>
     </row>
@@ -598,31 +612,34 @@
         <v>1998</v>
       </c>
       <c r="C5" t="n">
+        <v>41.9298782348633</v>
+      </c>
+      <c r="D5" t="n">
         <v>0.380236166897954</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
+        <v>5.1770268731498</v>
+      </c>
+      <c r="F5" t="n">
+        <v>584.448175174047</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6.37066811175281</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>22.6607423702209</v>
+      </c>
+      <c r="J5" t="n">
         <v>8.40223795613228</v>
       </c>
-      <c r="E5" t="n">
+      <c r="K5" t="n">
         <v>27.8800634028394</v>
       </c>
-      <c r="F5" t="n">
-        <v>22.6607423702209</v>
-      </c>
-      <c r="G5" t="n">
-        <v>5.1770268731498</v>
-      </c>
-      <c r="H5" t="n">
-        <v>584.448175174047</v>
-      </c>
-      <c r="I5" t="n">
-        <v>41.9298782348633</v>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>2.893</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>22.6195132518384</v>
       </c>
     </row>
@@ -636,31 +653,34 @@
         <v>1999</v>
       </c>
       <c r="C6" t="n">
+        <v>45.0674591064453</v>
+      </c>
+      <c r="D6" t="n">
         <v>0.350304290993083</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
+        <v>4.67015636882111</v>
+      </c>
+      <c r="F6" t="n">
+        <v>600.232323162952</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6.397316785543117</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="n">
+        <v>22.3758655367007</v>
+      </c>
+      <c r="J6" t="n">
         <v>6.10669589841958</v>
       </c>
-      <c r="E6" t="n">
+      <c r="K6" t="n">
         <v>28.3879405571158</v>
       </c>
-      <c r="F6" t="n">
-        <v>22.3758655367007</v>
-      </c>
-      <c r="G6" t="n">
-        <v>4.67015636882111</v>
-      </c>
-      <c r="H6" t="n">
-        <v>600.232323162952</v>
-      </c>
-      <c r="I6" t="n">
-        <v>45.0674591064453</v>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>3.088</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>22.957073677202</v>
       </c>
     </row>
@@ -674,33 +694,36 @@
         <v>2000</v>
       </c>
       <c r="C7" t="n">
+        <v>46.7210006713867</v>
+      </c>
+      <c r="D7" t="n">
         <v>0.525362089236087</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
+        <v>5.29329471892532</v>
+      </c>
+      <c r="F7" t="n">
+        <v>620.560472822105</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6.430623058110431</v>
+      </c>
+      <c r="H7" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="I7" t="n">
+        <v>22.2793826819325</v>
+      </c>
+      <c r="J7" t="n">
         <v>2.20825620937535</v>
       </c>
-      <c r="E7" t="n">
+      <c r="K7" t="n">
         <v>29.3217143619038</v>
       </c>
-      <c r="F7" t="n">
-        <v>22.2793826819325</v>
-      </c>
-      <c r="G7" t="n">
-        <v>5.29329471892532</v>
-      </c>
-      <c r="H7" t="n">
-        <v>620.560472822105</v>
-      </c>
-      <c r="I7" t="n">
-        <v>46.7210006713867</v>
-      </c>
-      <c r="J7" t="n">
-        <v>33.4</v>
-      </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>3.27</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>23.3145114975244</v>
       </c>
     </row>
@@ -714,31 +737,34 @@
         <v>2001</v>
       </c>
       <c r="C8" t="n">
+        <v>48.4609718322754</v>
+      </c>
+      <c r="D8" t="n">
         <v>0.145443904569924</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
+        <v>5.07728777526728</v>
+      </c>
+      <c r="F8" t="n">
+        <v>641.288922876274</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6.463480093085436</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>22.5838118742213</v>
+      </c>
+      <c r="J8" t="n">
         <v>2.0071737421384</v>
       </c>
-      <c r="E8" t="n">
+      <c r="K8" t="n">
         <v>32.0980170730117</v>
       </c>
-      <c r="F8" t="n">
-        <v>22.5838118742213</v>
-      </c>
-      <c r="G8" t="n">
-        <v>5.07728777526728</v>
-      </c>
-      <c r="H8" t="n">
-        <v>641.288922876274</v>
-      </c>
-      <c r="I8" t="n">
-        <v>48.4609718322754</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>3.609</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>23.6999214768623</v>
       </c>
     </row>
@@ -752,31 +778,34 @@
         <v>2002</v>
       </c>
       <c r="C9" t="n">
+        <v>49.6199493408203</v>
+      </c>
+      <c r="D9" t="n">
         <v>0.0955793676464671</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
+        <v>3.83312393993225</v>
+      </c>
+      <c r="F9" t="n">
+        <v>655.672139362272</v>
+      </c>
+      <c r="G9" t="n">
+        <v>6.485660876451147</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>22.8392543728467</v>
+      </c>
+      <c r="J9" t="n">
         <v>3.33256493271912</v>
       </c>
-      <c r="E9" t="n">
+      <c r="K9" t="n">
         <v>28.9673807211649</v>
       </c>
-      <c r="F9" t="n">
-        <v>22.8392543728467</v>
-      </c>
-      <c r="G9" t="n">
-        <v>3.83312393993225</v>
-      </c>
-      <c r="H9" t="n">
-        <v>655.672139362272</v>
-      </c>
-      <c r="I9" t="n">
-        <v>49.6199493408203</v>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>3.966</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>24.1132383547332</v>
       </c>
     </row>
@@ -790,31 +819,34 @@
         <v>2003</v>
       </c>
       <c r="C10" t="n">
+        <v>49.5259017944336</v>
+      </c>
+      <c r="D10" t="n">
         <v>0.44596078329809</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
+        <v>4.73956739963045</v>
+      </c>
+      <c r="F10" t="n">
+        <v>676.826252046427</v>
+      </c>
+      <c r="G10" t="n">
+        <v>6.517414596024433</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>22.4741487860882</v>
+      </c>
+      <c r="J10" t="n">
         <v>5.66870773441476</v>
       </c>
-      <c r="E10" t="n">
+      <c r="K10" t="n">
         <v>27.657884900158</v>
       </c>
-      <c r="F10" t="n">
-        <v>22.4741487860882</v>
-      </c>
-      <c r="G10" t="n">
-        <v>4.73956739963045</v>
-      </c>
-      <c r="H10" t="n">
-        <v>676.826252046427</v>
-      </c>
-      <c r="I10" t="n">
-        <v>49.5259017944336</v>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>4.32</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>24.5525557512625</v>
       </c>
     </row>
@@ -828,31 +860,34 @@
         <v>2004</v>
       </c>
       <c r="C11" t="n">
+        <v>46.3084297180176</v>
+      </c>
+      <c r="D11" t="n">
         <v>0.689472335587339</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
+        <v>5.23953291029852</v>
+      </c>
+      <c r="F11" t="n">
+        <v>702.656357081873</v>
+      </c>
+      <c r="G11" t="n">
+        <v>6.554867948800887</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>22.7797200060528</v>
+      </c>
+      <c r="J11" t="n">
         <v>7.58753638504689</v>
       </c>
-      <c r="E11" t="n">
+      <c r="K11" t="n">
         <v>26.8582341492431</v>
       </c>
-      <c r="F11" t="n">
-        <v>22.7797200060528</v>
-      </c>
-      <c r="G11" t="n">
-        <v>5.23953291029852</v>
-      </c>
-      <c r="H11" t="n">
-        <v>702.656357081873</v>
-      </c>
-      <c r="I11" t="n">
-        <v>46.3084297180176</v>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>4.316</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>25.0094809886101</v>
       </c>
     </row>
@@ -866,33 +901,36 @@
         <v>2005</v>
       </c>
       <c r="C12" t="n">
+        <v>45.1695098876953</v>
+      </c>
+      <c r="D12" t="n">
         <v>1.17065167448603</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
+        <v>6.53594493875502</v>
+      </c>
+      <c r="F12" t="n">
+        <v>739.203718353409</v>
+      </c>
+      <c r="G12" t="n">
+        <v>6.605573550554825</v>
+      </c>
+      <c r="H12" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>23.2998442190711</v>
+      </c>
+      <c r="J12" t="n">
         <v>7.04661816222038</v>
       </c>
-      <c r="E12" t="n">
+      <c r="K12" t="n">
         <v>34.396934864465</v>
       </c>
-      <c r="F12" t="n">
-        <v>23.2998442190711</v>
-      </c>
-      <c r="G12" t="n">
-        <v>6.53594493875502</v>
-      </c>
-      <c r="H12" t="n">
-        <v>739.203718353409</v>
-      </c>
-      <c r="I12" t="n">
-        <v>45.1695098876953</v>
-      </c>
-      <c r="J12" t="n">
-        <v>33.2</v>
-      </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>4.25</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>25.4769540701509</v>
       </c>
     </row>
@@ -906,31 +944,34 @@
         <v>2006</v>
       </c>
       <c r="C13" t="n">
+        <v>45.7007904052734</v>
+      </c>
+      <c r="D13" t="n">
         <v>0.635863899506714</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
+        <v>6.67190498576788</v>
+      </c>
+      <c r="F13" t="n">
+        <v>779.419570444998</v>
+      </c>
+      <c r="G13" t="n">
+        <v>6.658549502218567</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>24.0953205119221</v>
+      </c>
+      <c r="J13" t="n">
         <v>6.76526117054757</v>
       </c>
-      <c r="E13" t="n">
+      <c r="K13" t="n">
         <v>38.1119244325921</v>
       </c>
-      <c r="F13" t="n">
-        <v>24.0953205119221</v>
-      </c>
-      <c r="G13" t="n">
-        <v>6.67190498576788</v>
-      </c>
-      <c r="H13" t="n">
-        <v>779.419570444998</v>
-      </c>
-      <c r="I13" t="n">
-        <v>45.7007904052734</v>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>3.591</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>25.9479149992596</v>
       </c>
     </row>
@@ -944,31 +985,34 @@
         <v>2007</v>
       </c>
       <c r="C14" t="n">
+        <v>46.4658813476562</v>
+      </c>
+      <c r="D14" t="n">
         <v>0.817756922700044</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
+        <v>7.05859935449848</v>
+      </c>
+      <c r="F14" t="n">
+        <v>825.508229964537</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6.715999232982851</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>24.5005410079343</v>
+      </c>
+      <c r="J14" t="n">
         <v>9.106984969053819</v>
       </c>
-      <c r="E14" t="n">
+      <c r="K14" t="n">
         <v>39.9423826531735</v>
       </c>
-      <c r="F14" t="n">
-        <v>24.5005410079343</v>
-      </c>
-      <c r="G14" t="n">
-        <v>7.05859935449848</v>
-      </c>
-      <c r="H14" t="n">
-        <v>825.508229964537</v>
-      </c>
-      <c r="I14" t="n">
-        <v>46.4658813476562</v>
-      </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
         <v>4.015</v>
       </c>
-      <c r="L14" t="n">
+      <c r="M14" t="n">
         <v>26.415303779311</v>
       </c>
     </row>
@@ -982,31 +1026,34 @@
         <v>2008</v>
       </c>
       <c r="C15" t="n">
+        <v>44.5729598999023</v>
+      </c>
+      <c r="D15" t="n">
         <v>1.4496579161576</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
+        <v>6.01378975738535</v>
+      </c>
+      <c r="F15" t="n">
+        <v>866.45815762135</v>
+      </c>
+      <c r="G15" t="n">
+        <v>6.764413819035702</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>24.7270013036793</v>
+      </c>
+      <c r="J15" t="n">
         <v>8.90194489465153</v>
       </c>
-      <c r="E15" t="n">
+      <c r="K15" t="n">
         <v>42.6209140325589</v>
       </c>
-      <c r="F15" t="n">
-        <v>24.7270013036793</v>
-      </c>
-      <c r="G15" t="n">
-        <v>6.01378975738535</v>
-      </c>
-      <c r="H15" t="n">
-        <v>866.45815762135</v>
-      </c>
-      <c r="I15" t="n">
-        <v>44.5729598999023</v>
-      </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="n">
+      <c r="L15" t="n">
         <v>4.49</v>
       </c>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v>26.87206041368</v>
       </c>
     </row>
@@ -1020,31 +1067,34 @@
         <v>2009</v>
       </c>
       <c r="C16" t="n">
+        <v>48.1255798339844</v>
+      </c>
+      <c r="D16" t="n">
         <v>0.879517142536145</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
+        <v>5.04512479919337</v>
+      </c>
+      <c r="F16" t="n">
+        <v>901.729626251937</v>
+      </c>
+      <c r="G16" t="n">
+        <v>6.804314725962496</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>25.2955721814431</v>
+      </c>
+      <c r="J16" t="n">
         <v>5.42347236174679</v>
       </c>
-      <c r="E16" t="n">
+      <c r="K16" t="n">
         <v>40.092796223023</v>
       </c>
-      <c r="F16" t="n">
-        <v>25.2955721814431</v>
-      </c>
-      <c r="G16" t="n">
-        <v>5.04512479919337</v>
-      </c>
-      <c r="H16" t="n">
-        <v>901.729626251937</v>
-      </c>
-      <c r="I16" t="n">
-        <v>48.1255798339844</v>
-      </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>5</v>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>27.3111249057412</v>
       </c>
     </row>
@@ -1058,33 +1108,36 @@
         <v>2010</v>
       </c>
       <c r="C17" t="n">
+        <v>49.5031106793162</v>
+      </c>
+      <c r="D17" t="n">
         <v>1.06896766308322</v>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
+        <v>5.57178818533122</v>
+      </c>
+      <c r="F17" t="n">
+        <v>943.6642286423599</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6.849770412875309</v>
+      </c>
+      <c r="H17" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>24.9564767264585</v>
+      </c>
+      <c r="J17" t="n">
         <v>8.126676391699171</v>
       </c>
-      <c r="E17" t="n">
+      <c r="K17" t="n">
         <v>37.8028426708321</v>
       </c>
-      <c r="F17" t="n">
-        <v>24.9564767264585</v>
-      </c>
-      <c r="G17" t="n">
-        <v>5.57178818533122</v>
-      </c>
-      <c r="H17" t="n">
-        <v>943.6642286423599</v>
-      </c>
-      <c r="I17" t="n">
-        <v>49.5031106793162</v>
-      </c>
-      <c r="J17" t="n">
-        <v>32.1</v>
-      </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
         <v>3.379</v>
       </c>
-      <c r="L17" t="n">
+      <c r="M17" t="n">
         <v>27.7254372588696</v>
       </c>
     </row>
@@ -1098,31 +1151,34 @@
         <v>2011</v>
       </c>
       <c r="C18" t="n">
+        <v>49.7515496494472</v>
+      </c>
+      <c r="D18" t="n">
         <v>0.983399364184761</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
+        <v>6.46437912497728</v>
+      </c>
+      <c r="F18" t="n">
+        <v>995.579947155662</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6.903325428823803</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>25.0452996007551</v>
+      </c>
+      <c r="J18" t="n">
         <v>11.3951651552399</v>
       </c>
-      <c r="E18" t="n">
+      <c r="K18" t="n">
         <v>47.4208498356898</v>
       </c>
-      <c r="F18" t="n">
-        <v>25.0452996007551</v>
-      </c>
-      <c r="G18" t="n">
-        <v>6.46437912497728</v>
-      </c>
-      <c r="H18" t="n">
-        <v>995.579947155662</v>
-      </c>
-      <c r="I18" t="n">
-        <v>49.7515496494472</v>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="n">
+      <c r="L18" t="n">
         <v>3.737</v>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>28.1100162712427</v>
       </c>
     </row>
@@ -1136,31 +1192,34 @@
         <v>2012</v>
       </c>
       <c r="C19" t="n">
+        <v>51.6718482971191</v>
+      </c>
+      <c r="D19" t="n">
         <v>1.18850391920183</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
+        <v>6.52145877906443</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1050.39140404066</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6.956918139444686</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>25.3099593902625</v>
+      </c>
+      <c r="J19" t="n">
         <v>6.21750422069283</v>
       </c>
-      <c r="E19" t="n">
+      <c r="K19" t="n">
         <v>48.1109227490467</v>
       </c>
-      <c r="F19" t="n">
-        <v>25.3099593902625</v>
-      </c>
-      <c r="G19" t="n">
-        <v>6.52145877906443</v>
-      </c>
-      <c r="H19" t="n">
-        <v>1050.39140404066</v>
-      </c>
-      <c r="I19" t="n">
-        <v>51.6718482971191</v>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="n">
+      <c r="L19" t="n">
         <v>4.07</v>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v>28.4787972894576</v>
       </c>
     </row>
@@ -1174,31 +1233,34 @@
         <v>2013</v>
       </c>
       <c r="C20" t="n">
+        <v>55.6214332189314</v>
+      </c>
+      <c r="D20" t="n">
         <v>1.73532012481503</v>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
+        <v>6.01360565834344</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1103.15695907123</v>
+      </c>
+      <c r="G20" t="n">
+        <v>7.005931311098014</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>26.3070701636507</v>
+      </c>
+      <c r="J20" t="n">
         <v>7.53040640913172</v>
       </c>
-      <c r="E20" t="n">
+      <c r="K20" t="n">
         <v>46.2964027228174</v>
       </c>
-      <c r="F20" t="n">
-        <v>26.3070701636507</v>
-      </c>
-      <c r="G20" t="n">
-        <v>6.01360565834344</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1103.15695907123</v>
-      </c>
-      <c r="I20" t="n">
-        <v>55.6214332189314</v>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="n">
+      <c r="L20" t="n">
         <v>4.426</v>
       </c>
-      <c r="L20" t="n">
+      <c r="M20" t="n">
         <v>28.8407036106763</v>
       </c>
     </row>
@@ -1211,30 +1273,33 @@
       <c r="B21" t="n">
         <v>2014</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="n">
         <v>1.46870305074204</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
+        <v>6.0610593588495</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1159.40753475981</v>
+      </c>
+      <c r="G21" t="n">
+        <v>7.055664407728581</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>26.3110467833576</v>
+      </c>
+      <c r="J21" t="n">
         <v>6.99163889220848</v>
       </c>
-      <c r="E21" t="n">
+      <c r="K21" t="n">
         <v>44.5140801968096</v>
       </c>
-      <c r="F21" t="n">
-        <v>26.3110467833576</v>
-      </c>
-      <c r="G21" t="n">
-        <v>6.0610593588495</v>
-      </c>
-      <c r="H21" t="n">
-        <v>1159.40753475981</v>
-      </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="n">
+      <c r="L21" t="n">
         <v>4.417</v>
       </c>
-      <c r="L21" t="n">
+      <c r="M21" t="n">
         <v>29.1944442321013</v>
       </c>
     </row>
@@ -1248,31 +1313,34 @@
         <v>2015</v>
       </c>
       <c r="C22" t="n">
+        <v>59.4217414855957</v>
+      </c>
+      <c r="D22" t="n">
         <v>1.4507824552936</v>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
+        <v>6.55263987816197</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1224.38647668165</v>
+      </c>
+      <c r="G22" t="n">
+        <v>7.110195162156987</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>26.8313948329541</v>
+      </c>
+      <c r="J22" t="n">
         <v>6.19428022984983</v>
       </c>
-      <c r="E22" t="n">
+      <c r="K22" t="n">
         <v>42.0859963070382</v>
       </c>
-      <c r="F22" t="n">
-        <v>26.8313948329541</v>
-      </c>
-      <c r="G22" t="n">
-        <v>6.55263987816197</v>
-      </c>
-      <c r="H22" t="n">
-        <v>1224.38647668165</v>
-      </c>
-      <c r="I22" t="n">
-        <v>59.4217414855957</v>
-      </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="n">
+      <c r="L22" t="n">
         <v>4.397</v>
       </c>
-      <c r="L22" t="n">
+      <c r="M22" t="n">
         <v>29.5395099477892</v>
       </c>
     </row>
@@ -1286,33 +1354,36 @@
         <v>2016</v>
       </c>
       <c r="C23" t="n">
+        <v>64.1664546117285</v>
+      </c>
+      <c r="D23" t="n">
         <v>0.879528340271998</v>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
+        <v>7.11347821270093</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1299.83091360792</v>
+      </c>
+      <c r="G23" t="n">
+        <v>7.169989468534807</v>
+      </c>
+      <c r="H23" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="I23" t="n">
+        <v>31.0691513830358</v>
+      </c>
+      <c r="J23" t="n">
         <v>5.51352572692995</v>
       </c>
-      <c r="E23" t="n">
+      <c r="K23" t="n">
         <v>31.3341501346142</v>
       </c>
-      <c r="F23" t="n">
-        <v>31.0691513830358</v>
-      </c>
-      <c r="G23" t="n">
-        <v>7.11347821270093</v>
-      </c>
-      <c r="H23" t="n">
-        <v>1299.83091360792</v>
-      </c>
-      <c r="I23" t="n">
-        <v>64.1664546117285</v>
-      </c>
-      <c r="J23" t="n">
-        <v>32.4</v>
-      </c>
-      <c r="K23" t="n">
+      <c r="L23" t="n">
         <v>4.35</v>
       </c>
-      <c r="L23" t="n">
+      <c r="M23" t="n">
         <v>29.8753915517965</v>
       </c>
     </row>
@@ -1326,31 +1397,34 @@
         <v>2017</v>
       </c>
       <c r="C24" t="n">
+        <v>62.3408639225315</v>
+      </c>
+      <c r="D24" t="n">
         <v>0.616341784631384</v>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="n">
+        <v>6.59024999794057</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1373.75363740186</v>
+      </c>
+      <c r="G24" t="n">
+        <v>7.225302153504579</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>31.2482919641603</v>
+      </c>
+      <c r="J24" t="n">
         <v>5.70207015717238</v>
       </c>
-      <c r="E24" t="n">
+      <c r="K24" t="n">
         <v>29.9997306724343</v>
       </c>
-      <c r="F24" t="n">
-        <v>31.2482919641603</v>
-      </c>
-      <c r="G24" t="n">
-        <v>6.59024999794057</v>
-      </c>
-      <c r="H24" t="n">
-        <v>1373.75363740186</v>
-      </c>
-      <c r="I24" t="n">
-        <v>62.3408639225315</v>
-      </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="n">
+      <c r="L24" t="n">
         <v>4.372</v>
       </c>
-      <c r="L24" t="n">
+      <c r="M24" t="n">
         <v>30.2015798381799</v>
       </c>
     </row>
@@ -1364,31 +1438,34 @@
         <v>2018</v>
       </c>
       <c r="C25" t="n">
+        <v>65.2714888764112</v>
+      </c>
+      <c r="D25" t="n">
         <v>0.75354913412869</v>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="n">
+        <v>7.31941263014136</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1462.25050255713</v>
+      </c>
+      <c r="G25" t="n">
+        <v>7.287731968010632</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="n">
+        <v>31.9828135899766</v>
+      </c>
+      <c r="J25" t="n">
         <v>5.54362139486476</v>
       </c>
-      <c r="E25" t="n">
+      <c r="K25" t="n">
         <v>32.5146317240884</v>
       </c>
-      <c r="F25" t="n">
-        <v>31.9828135899766</v>
-      </c>
-      <c r="G25" t="n">
-        <v>7.31941263014136</v>
-      </c>
-      <c r="H25" t="n">
-        <v>1462.25050255713</v>
-      </c>
-      <c r="I25" t="n">
-        <v>65.2714888764112</v>
-      </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="n">
+      <c r="L25" t="n">
         <v>4.439</v>
       </c>
-      <c r="L25" t="n">
+      <c r="M25" t="n">
         <v>30.5175656009959</v>
       </c>
     </row>
@@ -1402,31 +1479,34 @@
         <v>2019</v>
       </c>
       <c r="C26" t="n">
+        <v>65.1185413488915</v>
+      </c>
+      <c r="D26" t="n">
         <v>0.543244141585063</v>
       </c>
-      <c r="D26" t="n">
+      <c r="E26" t="n">
+        <v>7.88191515117722</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1564.20802445636</v>
+      </c>
+      <c r="G26" t="n">
+        <v>7.355134920224906</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="n">
+        <v>32.8525491977868</v>
+      </c>
+      <c r="J26" t="n">
         <v>5.59199639930629</v>
       </c>
-      <c r="E26" t="n">
+      <c r="K26" t="n">
         <v>31.5780544912404</v>
       </c>
-      <c r="F26" t="n">
-        <v>32.8525491977868</v>
-      </c>
-      <c r="G26" t="n">
-        <v>7.88191515117722</v>
-      </c>
-      <c r="H26" t="n">
-        <v>1564.20802445636</v>
-      </c>
-      <c r="I26" t="n">
-        <v>65.1185413488915</v>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="n">
+      <c r="L26" t="n">
         <v>4.504</v>
       </c>
-      <c r="L26" t="n">
+      <c r="M26" t="n">
         <v>30.8228396343012</v>
       </c>
     </row>
@@ -1440,31 +1520,34 @@
         <v>2020</v>
       </c>
       <c r="C27" t="n">
+        <v>66.4329548486639</v>
+      </c>
+      <c r="D27" t="n">
         <v>0.407859894856915</v>
       </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
+        <v>3.44801755122445</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1604.6659234742</v>
+      </c>
+      <c r="G27" t="n">
+        <v>7.380670866530346</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="n">
+        <v>32.9115650824449</v>
+      </c>
+      <c r="J27" t="n">
         <v>5.69107474746211</v>
       </c>
-      <c r="E27" t="n">
+      <c r="K27" t="n">
         <v>26.271447376215</v>
       </c>
-      <c r="F27" t="n">
-        <v>32.9115650824449</v>
-      </c>
-      <c r="G27" t="n">
-        <v>3.44801755122445</v>
-      </c>
-      <c r="H27" t="n">
-        <v>1604.6659234742</v>
-      </c>
-      <c r="I27" t="n">
-        <v>66.4329548486639</v>
-      </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="n">
+      <c r="L27" t="n">
         <v>5.539</v>
       </c>
-      <c r="L27" t="n">
+      <c r="M27" t="n">
         <v>31.1168927321524</v>
       </c>
     </row>
@@ -1478,31 +1561,34 @@
         <v>2021</v>
       </c>
       <c r="C28" t="n">
+        <v>66.8282318620991</v>
+      </c>
+      <c r="D28" t="n">
         <v>0.414118154040593</v>
       </c>
-      <c r="D28" t="n">
+      <c r="E28" t="n">
+        <v>6.93867912442445</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1702.08028414189</v>
+      </c>
+      <c r="G28" t="n">
+        <v>7.439606478491974</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="n">
+        <v>33.3160943869001</v>
+      </c>
+      <c r="J28" t="n">
         <v>5.54565430773473</v>
       </c>
-      <c r="E28" t="n">
+      <c r="K28" t="n">
         <v>27.7240047036631</v>
       </c>
-      <c r="F28" t="n">
-        <v>33.3160943869001</v>
-      </c>
-      <c r="G28" t="n">
-        <v>6.93867912442445</v>
-      </c>
-      <c r="H28" t="n">
-        <v>1702.08028414189</v>
-      </c>
-      <c r="I28" t="n">
-        <v>66.8282318620991</v>
-      </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="n">
+      <c r="L28" t="n">
         <v>5.457</v>
       </c>
-      <c r="L28" t="n">
+      <c r="M28" t="n">
         <v>31.3992156886061</v>
       </c>
     </row>
@@ -1516,33 +1602,36 @@
         <v>2022</v>
       </c>
       <c r="C29" t="n">
+        <v>67.0384586440383</v>
+      </c>
+      <c r="D29" t="n">
         <v>0.347960024540439</v>
       </c>
-      <c r="D29" t="n">
+      <c r="E29" t="n">
+        <v>7.09982877575158</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1804.3493461776</v>
+      </c>
+      <c r="G29" t="n">
+        <v>7.49795533274916</v>
+      </c>
+      <c r="H29" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="I29" t="n">
+        <v>33.9200804971876</v>
+      </c>
+      <c r="J29" t="n">
         <v>7.69695437176898</v>
       </c>
-      <c r="E29" t="n">
+      <c r="K29" t="n">
         <v>33.7799672705735</v>
       </c>
-      <c r="F29" t="n">
-        <v>33.9200804971876</v>
-      </c>
-      <c r="G29" t="n">
-        <v>7.09982877575158</v>
-      </c>
-      <c r="H29" t="n">
-        <v>1804.3493461776</v>
-      </c>
-      <c r="I29" t="n">
-        <v>67.0384586440383</v>
-      </c>
-      <c r="J29" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="K29" t="n">
+      <c r="L29" t="n">
         <v>4.593</v>
       </c>
-      <c r="L29" t="n">
+      <c r="M29" t="n">
         <v>31.673734726234</v>
       </c>
     </row>
@@ -1556,31 +1645,34 @@
         <v>2023</v>
       </c>
       <c r="C30" t="n">
+        <v>65.9856598598849</v>
+      </c>
+      <c r="D30" t="n">
         <v>0.335721505298968</v>
       </c>
-      <c r="D30" t="n">
+      <c r="E30" t="n">
+        <v>5.77511237007889</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1885.37733613545</v>
+      </c>
+      <c r="G30" t="n">
+        <v>7.541883258170298</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="n">
+        <v>34.5942721606063</v>
+      </c>
+      <c r="J30" t="n">
         <v>9.883503037792099</v>
       </c>
-      <c r="E30" t="n">
+      <c r="K30" t="n">
         <v>30.9829714104596</v>
       </c>
-      <c r="F30" t="n">
-        <v>34.5942721606063</v>
-      </c>
-      <c r="G30" t="n">
-        <v>5.77511237007889</v>
-      </c>
-      <c r="H30" t="n">
-        <v>1885.37733613545</v>
-      </c>
-      <c r="I30" t="n">
-        <v>65.9856598598849</v>
-      </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="n">
+      <c r="L30" t="n">
         <v>3.352</v>
       </c>
-      <c r="L30" t="n">
+      <c r="M30" t="n">
         <v>32.1578465036834</v>
       </c>
     </row>
@@ -1594,31 +1686,34 @@
         <v>2024</v>
       </c>
       <c r="C31" t="n">
+        <v>64.2997191043961</v>
+      </c>
+      <c r="D31" t="n">
         <v>0.283870773350074</v>
       </c>
-      <c r="D31" t="n">
+      <c r="E31" t="n">
+        <v>4.22325911250161</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1941.27874360025</v>
+      </c>
+      <c r="G31" t="n">
+        <v>7.571102181101636</v>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="n">
+        <v>34.0971743458877</v>
+      </c>
+      <c r="J31" t="n">
         <v>10.4657482763412</v>
       </c>
-      <c r="E31" t="n">
+      <c r="K31" t="n">
         <v>26.7780758040478</v>
       </c>
-      <c r="F31" t="n">
-        <v>34.0971743458877</v>
-      </c>
-      <c r="G31" t="n">
-        <v>4.22325911250161</v>
-      </c>
-      <c r="H31" t="n">
-        <v>1941.27874360025</v>
-      </c>
-      <c r="I31" t="n">
-        <v>64.2997191043961</v>
-      </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="n">
+      <c r="L31" t="n">
         <v>3.635</v>
       </c>
-      <c r="L31" t="n">
+      <c r="M31" t="n">
         <v>32.6783196323307</v>
       </c>
     </row>
@@ -1639,10 +1734,11 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
-      <c r="K32" t="n">
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
         <v>3.778</v>
       </c>
-      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>